<commit_message>
docs: record V60 public stage verification and workbook delivery
</commit_message>
<xml_diff>
--- a/docs/THE_PIT_STAGES_V60_SUIVI.xlsx
+++ b/docs/THE_PIT_STAGES_V60_SUIVI.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stages" sheetId="1" r:id="Rc6a8797c73fd4e35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="2" r:id="R711d2bd865b04308"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stages" sheetId="1" r:id="R47ba91e4ae9a49f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="2" r:id="R136b2d09e8134c69"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -466,7 +466,8 @@
       </x:c>
       <x:c r="H4" s="12"/>
       <x:c r="I4" s="12" t="str">
-        <x:v>PUBLICATION : EN ATTENTE · aucune mise en ligne affirmée par ce classeur.</x:v>
+        <x:v>PUBLICATION VÉRIFIÉE · https://yautja-la-longue-chasse.vercel.app
+Révision : 56dc65cdc59ee371a9aa37773bde686132b95946</x:v>
       </x:c>
       <x:c r="J4" s="3"/>
       <x:c r="K4" s="3"/>
@@ -613,7 +614,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H10" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I10" s="3" t="str">
         <x:v>1. SUBSTITUTION : végétation originale. Faune conditionnée à une espèce vérifiée encore à produire.
@@ -661,7 +662,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H11" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I11" s="3" t="str">
         <x:v>1. Technicien adulte anonyme derrière une vitre ; tenue et salle adaptées, sans double de combattant.
@@ -708,7 +709,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H12" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I12" s="3" t="str">
         <x:v>1. SUBSTITUTION : treuil de carrière. Ouvriers aliens et espèce non validés, non produits.
@@ -754,7 +755,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H13" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I13" s="3" t="str">
         <x:v>1. PARTIEL : garde anonyme observant/saluant. Tirage pendant le round, pas de salut déclenché à la victoire.
@@ -802,7 +803,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H14" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I14" s="3" t="str">
         <x:v>1. Bras-outil et prothèse inerte ; mécanisme original, aucune arme spécifique attribuée.
@@ -849,7 +850,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H15" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I15" s="3" t="str">
         <x:v>1. Faune originale sur roche froide, sans espèce canonique ni immunité au feu affirmée.
@@ -895,7 +896,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H16" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I16" s="3" t="str">
         <x:v>1. Un drone à dôme lisse au plafond ; inspiration anatomique NECA, pas copie du Warrior de la référence.
@@ -943,7 +944,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H17" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I17" s="3" t="str">
         <x:v>1. Chariot de matériel original, roues animées ; aucun transport nommé certifié.
@@ -989,7 +990,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H18" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I18" s="3" t="str">
         <x:v>1. Patrouille adulte anonyme sur le quai ; pas d'évacuation narrative du quai simulée.
@@ -1036,7 +1037,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H19" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I19" s="3" t="str">
         <x:v>1. ADAPTATION : carrousel d'échantillons inspecté par un bras ; pas d'identification biologique canonique.
@@ -1083,7 +1084,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H20" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I20" s="3" t="str">
         <x:v>1. Adultes anonymes du décor nordique ; aucune identité, date ou arme de roster affirmée.
@@ -1130,7 +1131,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H21" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I21" s="3" t="str">
         <x:v>1. Gardes adultes anonymes sur chemin de ronde, équipement rangé ; pas de duel nommé.
@@ -1179,7 +1180,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H22" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I22" s="3" t="str">
         <x:v>1. CONDITION DE LIEU RESPECTÉE : cette variante est explicitement terrestre et originale ; caravane adulte anonyme.
@@ -1227,7 +1228,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H23" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I23" s="3" t="str">
         <x:v>1. Vague derrière la zone jouable, aucun effet physique sur les combattants.
@@ -1274,7 +1275,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H24" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I24" s="3" t="str">
         <x:v>1. Marins adultes anonymes et gestes de prudence ; pas de scénario de fuite persistant.
@@ -1322,7 +1323,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H25" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I25" s="3" t="str">
         <x:v>1. Oiseaux tropicaux sur perchoir ; aucune espèce ou tribu canonique inventée.
@@ -1369,7 +1370,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H26" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I26" s="3" t="str">
         <x:v>1. PARTIEL : annonceur anonyme au pupitre. Coupure de commentaire liée à l'apparition d'une menace non implémentée.
@@ -1416,7 +1417,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H27" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I27" s="3" t="str">
         <x:v>1. Captif adulte anonyme, hésitation/veille ; pas d'évasion ou d'objectif effectivement accompli.
@@ -1464,7 +1465,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H28" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I28" s="3" t="str">
         <x:v>1. Console de navigation originale ; pas d'état persistant d'évacuation simulé.
@@ -1511,7 +1512,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H29" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I29" s="3" t="str">
         <x:v>1. PARTIEL : un garde colonial adulte anonyme, pas une escouade humaine entière.
@@ -1557,7 +1558,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H30" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I30" s="3" t="str">
         <x:v>1. Aéronef d'après silhouette d'image officielle ; pas de fidélité absolue 1:1 ni d'armement inventé comme canon.
@@ -1604,7 +1605,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H31" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I31" s="3" t="str">
         <x:v>1. Quadrupède original du projet, aucune espèce canonique nommée.
@@ -1650,7 +1651,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H32" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I32" s="3" t="str">
         <x:v>1. ADAPTATION : archiviste examinant un objet, pas une calibration d'anneaux reproduite littéralement.
@@ -1696,7 +1697,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H33" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I33" s="3" t="str">
         <x:v>1. Instructeur adulte anonyme, posture d'observation/démonstration, lieu original.
@@ -1742,7 +1743,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H34" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="I34" s="3" t="str">
         <x:v>1. Quadrupède polaire original, aucune créature canonique ni planète attestée.
@@ -1787,7 +1788,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R654ea1ca92894102"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdc350c3797640b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2085,7 +2086,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O10" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P10" s="3" t="str">
         <x:v>3e8da646152a22911b37aa00cfce01c96c95f7e183d32a8c6b2566bc2984cbc9</x:v>
@@ -2135,7 +2136,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O11" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P11" s="3" t="str">
         <x:v>333f421e51fe557867c81d221b7e95f624cdfdb1b13c0e06e16af952dc9b9c43</x:v>
@@ -2185,7 +2186,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O12" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P12" s="3" t="str">
         <x:v>c949b7e72e7c90fd670d7df2fc4d51527b4c2ed20bb3615aeba0aeb9f93b2e04</x:v>
@@ -2235,7 +2236,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O13" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P13" s="3" t="str">
         <x:v>51a24c36f5f40ccfa7bfe43e2aae870e8445199c429103baf2e347fa61317ce1</x:v>
@@ -2285,7 +2286,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O14" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P14" s="3" t="str">
         <x:v>869f520cd260277846f800d86c8e667e7450d7fc3a8a08cf163f1dd121c0aa47</x:v>
@@ -2335,7 +2336,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O15" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P15" s="3" t="str">
         <x:v>b96e671fe89e97c2c01a04b803fa6f9d341e25355a4a0a7e0e13fc538031defc</x:v>
@@ -2385,7 +2386,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O16" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P16" s="3" t="str">
         <x:v>1047b5f38616ef37f3cf4d388acb0674a65c2291b533bd4ab52a5b0f95487308</x:v>
@@ -2435,7 +2436,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O17" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P17" s="3" t="str">
         <x:v>d87a8173b0b02fc1ea51c44136ec40069acacf2007eecc996a43ad85918ad267</x:v>
@@ -2485,7 +2486,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O18" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P18" s="3" t="str">
         <x:v>acefdebb5fae4a48ec00778418ea7e632a2d575dac3500854fdf02a9189918a2</x:v>
@@ -2535,7 +2536,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O19" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P19" s="3" t="str">
         <x:v>322fc5cc352738020aa741f09f4f93a1f1844af2e461f640c3a4f62f88822f04</x:v>
@@ -2585,7 +2586,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O20" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P20" s="3" t="str">
         <x:v>0e08187c7bfb5fb5588ea79542ce3d8655e86416c98d8a0144bedd6549ada174</x:v>
@@ -2635,7 +2636,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O21" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P21" s="3" t="str">
         <x:v>8d17ec1e9f1f248ad751ca88c2e3a5449f1522f3fb7d90398fc15f184eef4edc</x:v>
@@ -2685,7 +2686,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O22" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P22" s="3" t="str">
         <x:v>b37f6b9d27b50be3fdb2e98a485d9af79ef59f36c9b87b2c6cf536fbe9c6a1d3</x:v>
@@ -2735,7 +2736,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O23" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P23" s="3" t="str">
         <x:v>c8fd76d69fd5814c5cbb5f5643b0545d7d07f29ae0b0a8b6b545211055c8fc6c</x:v>
@@ -2785,7 +2786,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O24" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P24" s="3" t="str">
         <x:v>3dc86491e09d70e337db40454c0e61d9d4a413428d48423c3a36f1c77d0baae0</x:v>
@@ -2835,7 +2836,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O25" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P25" s="3" t="str">
         <x:v>32989ef1d1533116f969d50c260e21c63b788205b0f91a88b704f7af8336c9e7</x:v>
@@ -2885,7 +2886,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O26" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P26" s="3" t="str">
         <x:v>3072881125544d6e5adcbf7e4859d346a92e81611c8d16c2f4efdce8715b6a20</x:v>
@@ -2935,7 +2936,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O27" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P27" s="3" t="str">
         <x:v>a7afc2bb6d406f5e5da1154f905337267e01acad8a6a1d83d3996ca8b137e3df</x:v>
@@ -2985,7 +2986,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O28" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P28" s="3" t="str">
         <x:v>268636c2a77ad6b0022eadf6eeecc1819a03334b09a0e4e3ad8c047ad074f51f</x:v>
@@ -3035,7 +3036,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O29" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P29" s="3" t="str">
         <x:v>a1b777e424894f174fba192d27e5a14f89d8ef0db11ce50912a498e21238918d</x:v>
@@ -3085,7 +3086,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O30" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P30" s="3" t="str">
         <x:v>7c62d418fea06ea2ce1f5c1a8fe841cf1b2f3fd9e1016e97197702b258ed8bcd</x:v>
@@ -3135,7 +3136,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O31" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P31" s="3" t="str">
         <x:v>d7e1024ccbd9096dd39fc93e20d932313d2f3271521c24573412c90adbf54783</x:v>
@@ -3185,7 +3186,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O32" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P32" s="3" t="str">
         <x:v>e718703fd439caeb9b19c6e9952b8625889e5e733c79876d7e47bb2e98b9b54e</x:v>
@@ -3235,7 +3236,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O33" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P33" s="3" t="str">
         <x:v>540d402cfcf9ea8d9c5ef06d752dae6ea644b76d96e855a3d5d1294a596a2ddf</x:v>
@@ -3285,7 +3286,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O34" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P34" s="3" t="str">
         <x:v>7cad0b6fc4a19d843a145bcf0316bd152451da58288809d94dd50ebd5f0e0ae5</x:v>
@@ -3335,7 +3336,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O35" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P35" s="3" t="str">
         <x:v>2ccc3ea9ecd20e07465a9462309dfa877a9d89d02ab6164ea31c11c6128355e2</x:v>
@@ -3385,7 +3386,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O36" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P36" s="3" t="str">
         <x:v>d29f194539cd942be5297cb2d48ab1c16f5a7a03665ffe7ce0742dc5f652e0b7</x:v>
@@ -3435,7 +3436,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O37" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P37" s="3" t="str">
         <x:v>fa771c0839343a4ee4608285c9661938ed3530e7cf4d6ffd280a58769527b4a8</x:v>
@@ -3485,7 +3486,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O38" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P38" s="3" t="str">
         <x:v>b2b50f83cdd4b6aa994081d980815fb78562e26975e1d765792254a839a0824c</x:v>
@@ -3535,7 +3536,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O39" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P39" s="3" t="str">
         <x:v>e894f427b51f6e5a599b4bf7b0a185c85eef6ef44c6b4b876f9bd08b9edca7c6</x:v>
@@ -3585,7 +3586,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O40" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P40" s="3" t="str">
         <x:v>964e0ff66f03e7ef431a78eee6640cb6fc1b85dfd24a18e7b87ee43a77c0d529</x:v>
@@ -3635,7 +3636,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O41" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P41" s="3" t="str">
         <x:v>19e39bbdde270a026bc330e824f8e65ca33b35bfd88c582a93b7e41c5dfb4e74</x:v>
@@ -3685,7 +3686,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O42" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P42" s="3" t="str">
         <x:v>f76211d7ee9623e024499ba95f13b988e2b192dd9c775777c41a496d71154697</x:v>
@@ -3735,7 +3736,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O43" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P43" s="3" t="str">
         <x:v>e2756de56ecb84713d0eb398c506cd4eac7ba9f7745b8d5033f09f743dc14d06</x:v>
@@ -3785,7 +3786,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O44" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P44" s="3" t="str">
         <x:v>6505d70a2f8555f4149bd199f79b2a79d32c9ef77348e75ef1945fa2c5555bcd</x:v>
@@ -3835,7 +3836,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O45" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P45" s="3" t="str">
         <x:v>06e15f6ab586c6db257cda82245aa0d18967d9844aa6ea2e4c403aa9863d7587</x:v>
@@ -3885,7 +3886,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O46" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P46" s="3" t="str">
         <x:v>8d0a3aa0b98d86dcc42483d22b1fc290e6b0e817538d025c801fffefa6925d59</x:v>
@@ -3935,7 +3936,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O47" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P47" s="3" t="str">
         <x:v>a6c82685a899ccbf690d2c6bb82540bf8e458953e1393ce8b8ba535bd8409333</x:v>
@@ -3985,7 +3986,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O48" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P48" s="3" t="str">
         <x:v>80f2ec37b415b26b5465a7d77c7e2da72088b2cf1af5f6385ad693256278a24a</x:v>
@@ -4035,7 +4036,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O49" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P49" s="3" t="str">
         <x:v>a7fe46afee07dcc120a19b5759723772749b6f8210515bc353936b6bc89a34ba</x:v>
@@ -4085,7 +4086,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O50" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P50" s="3" t="str">
         <x:v>32896b1fd8a8976a49dcae9cc94f2fedb2d0fa7c9c35ace4328ecf2f30f04197</x:v>
@@ -4135,7 +4136,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O51" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P51" s="3" t="str">
         <x:v>2e112a613857af91d0712b1cd2d4a16e3bd85b84f8ad1ce352cc4ceea2e51bd8</x:v>
@@ -4185,7 +4186,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O52" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P52" s="3" t="str">
         <x:v>cb90e3430ded0f3a3a74d52b3efe0a9d303b4206adcc58d563244b71ff63ff32</x:v>
@@ -4235,7 +4236,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O53" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P53" s="3" t="str">
         <x:v>582a2ac307666b012ddc35100c1659666d4220c243b84a3270ba70d8fba5e0d7</x:v>
@@ -4285,7 +4286,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O54" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P54" s="3" t="str">
         <x:v>8bb4451f7222417d8a48f2d3c1e6a224ba1b9ff4cf332d895ae0f951a8c63cc5</x:v>
@@ -4335,7 +4336,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O55" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P55" s="3" t="str">
         <x:v>3a8fc8c697b92c0581198ef54fcbe79007ed857f63524902f7d167a998284884</x:v>
@@ -4385,7 +4386,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O56" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P56" s="3" t="str">
         <x:v>7fc6ad7aeb9a9bac12f352abe1f69173da0537b2b54bf41cef12ec57f642d873</x:v>
@@ -4435,7 +4436,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O57" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P57" s="3" t="str">
         <x:v>42a55b867a5b9354ce6ee198b90a4836789ebfb7d1a20b683704d428edf809cb</x:v>
@@ -4485,7 +4486,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O58" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P58" s="3" t="str">
         <x:v>e72c6a3062712e76c4551e21e091ec76601bc540f8b565e31fdecdf5fe6d662b</x:v>
@@ -4535,7 +4536,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O59" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P59" s="3" t="str">
         <x:v>d45b3798a4d385dc36362e5014a4dfb6ccaec04ce35b7d0fdb9cfd6c2c8f315c</x:v>
@@ -4585,7 +4586,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O60" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P60" s="3" t="str">
         <x:v>0926b4c735dbf0ce21498a205c2ca19e75fa6ff0fee15535658134bfc8c800a2</x:v>
@@ -4635,7 +4636,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O61" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P61" s="3" t="str">
         <x:v>8307ee95585af1322062a9329f4aae32d1ba86ac7f573eff4cba38e9e111c598</x:v>
@@ -4685,7 +4686,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O62" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P62" s="3" t="str">
         <x:v>a0b695020a13e1b8274d887fc0045c64a7fcdf30985982ff8fc1d9f8ea11badd</x:v>
@@ -4735,7 +4736,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O63" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P63" s="3" t="str">
         <x:v>d89c1cb01bbdece003eb266bea397f9b3e584446e69de6c6408e1c4112a641f5</x:v>
@@ -4785,7 +4786,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O64" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P64" s="3" t="str">
         <x:v>33a067c44ac096031f20d18ce2462252696e4e2a2a186c538a532297a24bef06</x:v>
@@ -4835,7 +4836,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O65" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P65" s="3" t="str">
         <x:v>d604a471a7e8267ad928dcc01cac792ea3c4e90a8f98781a0e8d15473026b3bc</x:v>
@@ -4885,7 +4886,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O66" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P66" s="3" t="str">
         <x:v>6142e041393debe62742aa7543d22d9bed000aaaae9245c8d434ff6b1edff67a</x:v>
@@ -4935,7 +4936,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O67" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P67" s="3" t="str">
         <x:v>7bbd2fa182ba32c89ed615eacfb26f8f7b61fa4d5fe2b2323947a9fe7ed89077</x:v>
@@ -4985,7 +4986,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O68" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P68" s="3" t="str">
         <x:v>2cf15f6bce5ab328d2712131ea165841cc0518e6729987b359816891923d805e</x:v>
@@ -5035,7 +5036,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O69" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P69" s="3" t="str">
         <x:v>549678c930a2442839cae7a2ec1b378c86fa4185d6a79a0efbf89acf1cfc1adb</x:v>
@@ -5085,7 +5086,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O70" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P70" s="3" t="str">
         <x:v>08b7dbe616178ba1ffd82f73eaac97f66ccf1c7ed467a689b6a9b214525cd924</x:v>
@@ -5135,7 +5136,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O71" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P71" s="3" t="str">
         <x:v>91bf5233f37b3cb1a4d7c44c72ee86d949f658f7102af26a0dffa584f7389fb4</x:v>
@@ -5185,7 +5186,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O72" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P72" s="3" t="str">
         <x:v>65955686497ad660a95c676cd3b453f4d6e1dae411764cee323c2bda944c889d</x:v>
@@ -5235,7 +5236,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O73" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P73" s="3" t="str">
         <x:v>ad6a925ef9a737d641fb75cdf80f79bbf630f94176ab687831a0e8e9fba8d1c1</x:v>
@@ -5285,7 +5286,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O74" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P74" s="3" t="str">
         <x:v>21d7e321a9da629f5ec5f9ff3a5c24176bd49148413071be81b636033f37f9db</x:v>
@@ -5335,7 +5336,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O75" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P75" s="3" t="str">
         <x:v>7314f950bc9fc77213018123aa83002a6ee499012a7b2541425b8de2046de430</x:v>
@@ -5385,7 +5386,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O76" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P76" s="3" t="str">
         <x:v>14839bd74013b3b74c5a81f988432a4cb1de7c768018ebc55d88c1500e8431fd</x:v>
@@ -5435,7 +5436,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O77" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P77" s="3" t="str">
         <x:v>9c6998f137b540101d9f78ecb2ff35426402551d8270430f456399fb7d439b1c</x:v>
@@ -5485,7 +5486,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O78" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P78" s="3" t="str">
         <x:v>86a22c38a794d5af03e828a4d268e12b264e73a45241e8b5ffd1fefd3edc3a26</x:v>
@@ -5535,7 +5536,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O79" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P79" s="3" t="str">
         <x:v>c277ea9bdf08660e50d2dc375d8a609293e46dca9f4d38e6fe7db760f944b978</x:v>
@@ -5585,7 +5586,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O80" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P80" s="3" t="str">
         <x:v>faca049c5300c4ea49324e406fafe8688d78033630f186f0b5b77037d48cdce3</x:v>
@@ -5635,7 +5636,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O81" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P81" s="3" t="str">
         <x:v>199598916ffba1e3ec8335d007d357b2f6c74e0a556ef38ca175d427a4d42601</x:v>
@@ -5685,7 +5686,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O82" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P82" s="3" t="str">
         <x:v>c64a45146145a70542102d2d948791575314ef3fa6099066dd36d51ce25f99cf</x:v>
@@ -5735,7 +5736,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O83" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P83" s="3" t="str">
         <x:v>19cfb08e9f32b943089ff89d5b5bbb4895dcb7795e671b627e7d80b4ee044508</x:v>
@@ -5785,7 +5786,7 @@
         <x:v>1536 × 1024 px ; 3 dessins/s</x:v>
       </x:c>
       <x:c r="O84" s="16" t="str">
-        <x:v>EN ATTENTE</x:v>
+        <x:v>PUBLIÉE · PREUVE VÉRIFIÉE</x:v>
       </x:c>
       <x:c r="P84" s="3" t="str">
         <x:v>040657613715cfb3577723fc9baafaf6f4563ca4bc5c4f0cce35c9c85d19181e</x:v>
@@ -5813,7 +5814,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raed0df9e9d804d9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f500d4d4b2048ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>